<commit_message>
Deployed b149f6a with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/campus_connect-gantt-chart_ms.xlsx
+++ b/campus_connect-gantt-chart_ms.xlsx
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="E3" s="55" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="F3" s="53" t="n"/>
     </row>
@@ -3462,10 +3462,20 @@
           <t>Task 3.1 — NextAuth API Route (src/app/api/auth/[...nextauth]/route.ts)</t>
         </is>
       </c>
-      <c r="C29" s="39" t="n"/>
-      <c r="D29" s="20" t="n"/>
-      <c r="E29" s="57" t="n"/>
-      <c r="F29" s="58" t="n"/>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="57" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F29" s="58" t="n">
+        <v>46275</v>
+      </c>
       <c r="G29" s="16" t="n"/>
       <c r="H29" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -3535,10 +3545,20 @@
           <t>Task 3.2 — Register API (src/app/api/register/route.ts)</t>
         </is>
       </c>
-      <c r="C30" s="39" t="n"/>
-      <c r="D30" s="20" t="n"/>
-      <c r="E30" s="57" t="n"/>
-      <c r="F30" s="58" t="n"/>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="57" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F30" s="58" t="n">
+        <v>46275</v>
+      </c>
       <c r="G30" s="16" t="n"/>
       <c r="H30" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -3608,10 +3628,20 @@
           <t>Task 3.3 — Auth Pages UI (Layout, Login, Register, Verify)</t>
         </is>
       </c>
-      <c r="C31" s="39" t="n"/>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="57" t="n"/>
-      <c r="F31" s="58" t="n"/>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="57" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>46276</v>
+      </c>
       <c r="G31" s="16" t="n"/>
       <c r="H31" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -3681,10 +3711,20 @@
           <t>Task 3.4 — Session Provider Wrapper (src/app/layout.tsx)</t>
         </is>
       </c>
-      <c r="C32" s="39" t="n"/>
-      <c r="D32" s="20" t="n"/>
-      <c r="E32" s="57" t="n"/>
-      <c r="F32" s="58" t="n"/>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="57" t="n">
+        <v>46276</v>
+      </c>
+      <c r="F32" s="58" t="n">
+        <v>46276</v>
+      </c>
       <c r="G32" s="16" t="n"/>
       <c r="H32" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -3754,10 +3794,20 @@
           <t>Task 3.5 — Invite Link System (src/app/api/admin/invite/route.ts)</t>
         </is>
       </c>
-      <c r="C33" s="39" t="n"/>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="57" t="n"/>
-      <c r="F33" s="58" t="n"/>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="57" t="n">
+        <v>46276</v>
+      </c>
+      <c r="F33" s="58" t="n">
+        <v>46276</v>
+      </c>
       <c r="G33" s="16" t="n"/>
       <c r="H33" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -3900,10 +3950,20 @@
           <t>Task 4.1 — Dashboard Layout (src/app/(dashboard)/layout.tsx)</t>
         </is>
       </c>
-      <c r="C35" s="39" t="n"/>
-      <c r="D35" s="20" t="n"/>
-      <c r="E35" s="57" t="n"/>
-      <c r="F35" s="58" t="n"/>
+      <c r="C35" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D35" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="57" t="n">
+        <v>46277</v>
+      </c>
+      <c r="F35" s="58" t="n">
+        <v>46277</v>
+      </c>
       <c r="G35" s="16" t="n"/>
       <c r="H35" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -3973,10 +4033,20 @@
           <t>Task 4.2 — Profile Page &amp; API (src/app/api/users/[id])</t>
         </is>
       </c>
-      <c r="C36" s="39" t="n"/>
-      <c r="D36" s="20" t="n"/>
-      <c r="E36" s="57" t="n"/>
-      <c r="F36" s="58" t="n"/>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D36" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="57" t="n">
+        <v>46277</v>
+      </c>
+      <c r="F36" s="58" t="n">
+        <v>46278</v>
+      </c>
       <c r="G36" s="16" t="n"/>
       <c r="H36" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4046,10 +4116,20 @@
           <t>Task 4.3 — Friend System API &amp; UI (src/app/api/friends)</t>
         </is>
       </c>
-      <c r="C37" s="39" t="n"/>
-      <c r="D37" s="20" t="n"/>
-      <c r="E37" s="57" t="n"/>
-      <c r="F37" s="58" t="n"/>
+      <c r="C37" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D37" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="57" t="n">
+        <v>46277</v>
+      </c>
+      <c r="F37" s="58" t="n">
+        <v>46278</v>
+      </c>
       <c r="G37" s="16" t="n"/>
       <c r="H37" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4119,10 +4199,20 @@
           <t>Task 4.4 — Social Feed API &amp; UI (src/app/api/posts)</t>
         </is>
       </c>
-      <c r="C38" s="39" t="n"/>
-      <c r="D38" s="20" t="n"/>
-      <c r="E38" s="57" t="n"/>
-      <c r="F38" s="58" t="n"/>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D38" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="57" t="n">
+        <v>46278</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>46278</v>
+      </c>
       <c r="G38" s="16" t="n"/>
       <c r="H38" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4265,10 +4355,20 @@
           <t>Task 5.1 — Groups API (src/app/api/groups)</t>
         </is>
       </c>
-      <c r="C40" s="39" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="57" t="n"/>
-      <c r="F40" s="58" t="n"/>
+      <c r="C40" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D40" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="57" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F40" s="58" t="n">
+        <v>46279</v>
+      </c>
       <c r="G40" s="16" t="n"/>
       <c r="H40" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4338,10 +4438,20 @@
           <t>Task 5.2 — Group Pages UI (Grid, Feed, Members)</t>
         </is>
       </c>
-      <c r="C41" s="39" t="n"/>
-      <c r="D41" s="20" t="n"/>
-      <c r="E41" s="57" t="n"/>
-      <c r="F41" s="58" t="n"/>
+      <c r="C41" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="57" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F41" s="58" t="n">
+        <v>46279</v>
+      </c>
       <c r="G41" s="16" t="n"/>
       <c r="H41" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4411,10 +4521,20 @@
           <t>Task 5.3 — Course Materials API (src/app/api/groups/[id]/materials)</t>
         </is>
       </c>
-      <c r="C42" s="39" t="n"/>
-      <c r="D42" s="42" t="n"/>
-      <c r="E42" s="57" t="n"/>
-      <c r="F42" s="58" t="n"/>
+      <c r="C42" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D42" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="57" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F42" s="58" t="n">
+        <v>46279</v>
+      </c>
       <c r="G42" s="16" t="n"/>
       <c r="H42" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4484,10 +4604,20 @@
           <t>Task 5.4 — Course Materials UI (FileUploader &amp; PdfViewerModal)</t>
         </is>
       </c>
-      <c r="C43" s="39" t="n"/>
-      <c r="D43" s="42" t="n"/>
-      <c r="E43" s="57" t="n"/>
-      <c r="F43" s="58" t="n"/>
+      <c r="C43" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D43" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="57" t="n">
+        <v>46279</v>
+      </c>
+      <c r="F43" s="58" t="n">
+        <v>46279</v>
+      </c>
       <c r="G43" s="16" t="n"/>
       <c r="H43" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>

</xml_diff>

<commit_message>
Deployed 2e55f27 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/campus_connect-gantt-chart_ms.xlsx
+++ b/campus_connect-gantt-chart_ms.xlsx
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="E3" s="55" t="n">
-        <v>46279</v>
+        <v>46306</v>
       </c>
       <c r="F3" s="53" t="n"/>
     </row>
@@ -4760,10 +4760,20 @@
           <t>Task 6.1 — Events API (src/app/api/events)</t>
         </is>
       </c>
-      <c r="C45" s="39" t="n"/>
-      <c r="D45" s="42" t="n"/>
-      <c r="E45" s="57" t="n"/>
-      <c r="F45" s="58" t="n"/>
+      <c r="C45" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D45" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="57" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F45" s="58" t="n">
+        <v>46300</v>
+      </c>
       <c r="G45" s="16" t="n"/>
       <c r="H45" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4833,10 +4843,20 @@
           <t>Task 6.2 — Schedule UI (CalendarView &amp; EventModal)</t>
         </is>
       </c>
-      <c r="C46" s="39" t="n"/>
-      <c r="D46" s="42" t="n"/>
-      <c r="E46" s="57" t="n"/>
-      <c r="F46" s="58" t="n"/>
+      <c r="C46" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D46" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="57" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F46" s="58" t="n">
+        <v>46301</v>
+      </c>
       <c r="G46" s="16" t="n"/>
       <c r="H46" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4906,10 +4926,20 @@
           <t>Task 6.3 — Event Notifications &amp; Socket Broadcast</t>
         </is>
       </c>
-      <c r="C47" s="39" t="n"/>
-      <c r="D47" s="42" t="n"/>
-      <c r="E47" s="57" t="n"/>
-      <c r="F47" s="58" t="n"/>
+      <c r="C47" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D47" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="57" t="n">
+        <v>46301</v>
+      </c>
+      <c r="F47" s="58" t="n">
+        <v>46301</v>
+      </c>
       <c r="G47" s="16" t="n"/>
       <c r="H47" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5052,10 +5082,20 @@
           <t>Task 7.1 — Custom Server Setup (server.ts with Socket.io)</t>
         </is>
       </c>
-      <c r="C49" s="39" t="n"/>
-      <c r="D49" s="42" t="n"/>
-      <c r="E49" s="57" t="n"/>
-      <c r="F49" s="58" t="n"/>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D49" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="57" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F49" s="58" t="n">
+        <v>46302</v>
+      </c>
       <c r="G49" s="16" t="n"/>
       <c r="H49" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5125,10 +5165,20 @@
           <t>Task 7.2 — Messaging API (src/app/api/messages)</t>
         </is>
       </c>
-      <c r="C50" s="39" t="n"/>
-      <c r="D50" s="42" t="n"/>
-      <c r="E50" s="57" t="n"/>
-      <c r="F50" s="58" t="n"/>
+      <c r="C50" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D50" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="57" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F50" s="58" t="n">
+        <v>46303</v>
+      </c>
       <c r="G50" s="16" t="n"/>
       <c r="H50" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5198,10 +5248,20 @@
           <t>Task 7.3 — Messaging UI (UserChatList &amp; ChatBox)</t>
         </is>
       </c>
-      <c r="C51" s="39" t="n"/>
-      <c r="D51" s="42" t="n"/>
-      <c r="E51" s="57" t="n"/>
-      <c r="F51" s="58" t="n"/>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D51" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="57" t="n">
+        <v>46303</v>
+      </c>
+      <c r="F51" s="58" t="n">
+        <v>46304</v>
+      </c>
       <c r="G51" s="16" t="n"/>
       <c r="H51" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5271,10 +5331,20 @@
           <t>Task 7.4 — Notifications API (src/app/api/notifications)</t>
         </is>
       </c>
-      <c r="C52" s="39" t="n"/>
-      <c r="D52" s="42" t="n"/>
-      <c r="E52" s="57" t="n"/>
-      <c r="F52" s="58" t="n"/>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D52" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="57" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F52" s="58" t="n">
+        <v>46305</v>
+      </c>
       <c r="G52" s="16" t="n"/>
       <c r="H52" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5344,10 +5414,20 @@
           <t>Task 7.5 — Notification Bell UI (NotificationDropdown.tsx)</t>
         </is>
       </c>
-      <c r="C53" s="39" t="n"/>
-      <c r="D53" s="42" t="n"/>
-      <c r="E53" s="57" t="n"/>
-      <c r="F53" s="58" t="n"/>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D53" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="57" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F53" s="58" t="n">
+        <v>46305</v>
+      </c>
       <c r="G53" s="16" t="n"/>
       <c r="H53" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5490,10 +5570,20 @@
           <t>Task 8.1 — Admin API Routes (Users, Settings, Reports)</t>
         </is>
       </c>
-      <c r="C55" s="39" t="n"/>
-      <c r="D55" s="42" t="n"/>
-      <c r="E55" s="57" t="n"/>
-      <c r="F55" s="58" t="n"/>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D55" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="57" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F55" s="58" t="n">
+        <v>46306</v>
+      </c>
       <c r="G55" s="16" t="n"/>
       <c r="H55" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>

</xml_diff>